<commit_message>
Updated POL_grids_syn_5 model - 2025-11-12 17:46
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_syn_5/Sets-vervestacks.xlsx
+++ b/VerveStacks_POL_grids_syn_5/Sets-vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4828C01F-0644-4BDA-A765-A37E9D2351D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{448C175B-982D-4168-A252-3EBEB65E190C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -106,12 +106,6 @@
     <t>Supercritical Coal</t>
   </si>
   <si>
-    <t>ep_gas_internal_combustion*,ep_oil_internal_combustion*</t>
-  </si>
-  <si>
-    <t>ep_gas_steam_turbine*,ep_oil_steam_turbine*</t>
-  </si>
-  <si>
     <t>STG</t>
   </si>
   <si>
@@ -124,24 +118,9 @@
     <t>IGCC</t>
   </si>
   <si>
-    <t>ep_bioenergy*,bioen*</t>
-  </si>
-  <si>
-    <t>ep_gas_combined_cycle*,ep_oil_combined_cycle*,CCGT*,*GasCC*</t>
-  </si>
-  <si>
-    <t>ep_gas_gas_turbine*,ep_oil_gas_turbine*,gas turbine*,EN*CT*</t>
-  </si>
-  <si>
-    <t>ep_coal_CFB*,ep_coal_subcritical*,*subcritical*</t>
-  </si>
-  <si>
     <t>*IGCC*</t>
   </si>
   <si>
-    <t>ep_coal_supercritical*,ep_coal_supercritical_CCS*,ep_coal_ultra-supercritical*,ep_coal_ultra-supercritical_CCS*,*supercritical*</t>
-  </si>
-  <si>
     <t>Gas_Oil Steam</t>
   </si>
   <si>
@@ -332,6 +311,27 @@
   </si>
   <si>
     <t>distr*</t>
+  </si>
+  <si>
+    <t>e*[_]gas_combined_cycle*,e*[_]oil_combined_cycle*,CCGT*,*GasCC*</t>
+  </si>
+  <si>
+    <t>e*[_]gas_internal_combustion*,e*[_]oil_internal_combustion*</t>
+  </si>
+  <si>
+    <t>e*[_]gas_steam_turbine*,e*[_]oil_steam_turbine*</t>
+  </si>
+  <si>
+    <t>e*[_]gas_gas_turbine*,e*[_]oil_gas_turbine*,gas turbine*,EN*CT*</t>
+  </si>
+  <si>
+    <t>e*[_]coal_CFB*,e*[_]coal_subcritical*,*subcritical*</t>
+  </si>
+  <si>
+    <t>e*[_]coal_supercritical*,e*[_]coal_supercritical_CCS*,e*[_]coal_ultra-supercritical*,e*[_]coal_ultra-supercritical_CCS*,*supercritical*</t>
+  </si>
+  <si>
+    <t>e*[_]bioenergy*,bioen*</t>
   </si>
   <si>
     <t>~tfm_psets</t>
@@ -1722,39 +1722,39 @@
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D25" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="D26" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D28" t="str">
         <f>B28</f>
@@ -1763,7 +1763,7 @@
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B29" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="D29" t="str">
         <f>B29</f>
@@ -1772,7 +1772,7 @@
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D30" t="str">
         <f>B30</f>
@@ -1781,7 +1781,7 @@
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D31" t="str">
         <f>B31</f>
@@ -1790,39 +1790,39 @@
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B32" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="D32" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B33" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="D33" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B34" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="D34" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B35" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D35" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B36" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D36" t="str">
         <f>B36</f>
@@ -1831,7 +1831,7 @@
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B37" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D37" t="str">
         <f>B37</f>
@@ -1847,7 +1847,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E20B5D50-ABF7-427D-B8E7-30C4499E062E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4166D441-BA5B-4FFE-A564-02B20AA8B06E}">
   <dimension ref="B9:E120"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -3466,7 +3466,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
-        <v>29</v>
+        <v>91</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -3475,45 +3475,45 @@
         <v>18</v>
       </c>
       <c r="H3" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="I3" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>22</v>
+        <v>92</v>
       </c>
       <c r="F4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>23</v>
+        <v>93</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="F6" t="s">
         <v>19</v>
       </c>
       <c r="H6" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="I6" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>31</v>
+        <v>95</v>
       </c>
       <c r="F7" t="s">
         <v>20</v>
@@ -3521,7 +3521,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>33</v>
+        <v>96</v>
       </c>
       <c r="F8" t="s">
         <v>21</v>
@@ -3529,57 +3529,57 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>28</v>
+        <v>97</v>
       </c>
       <c r="F10" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D11" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="F11" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B12" s="3"/>
       <c r="D12" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="F12" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="G12" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D13" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G13" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D14" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.45">
@@ -3587,13 +3587,13 @@
         <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="F15" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.45">
@@ -3601,121 +3601,121 @@
         <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="F16" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.45">
       <c r="B17" s="3" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D17" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="H17" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="I17" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="D18" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F18" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" t="s">
         <v>24</v>
-      </c>
-      <c r="B19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F19" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="F20" t="s">
+        <v>30</v>
+      </c>
+      <c r="H20" t="s">
         <v>37</v>
       </c>
-      <c r="H20" t="s">
-        <v>44</v>
-      </c>
       <c r="I20" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F21" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="B22" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="F22" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="F23" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F24" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="B25" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="F25" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.45">
@@ -3993,18 +3993,18 @@
     </row>
     <row r="47" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B47" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="F47" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B48" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="F48" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_syn_5 model - 2025-11-19 13:12
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_syn_5/Sets-vervestacks.xlsx
+++ b/VerveStacks_POL_grids_syn_5/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{448C175B-982D-4168-A252-3EBEB65E190C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F59C74D8-47EC-47EC-9329-4807F30D3FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1847,7 +1847,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4166D441-BA5B-4FFE-A564-02B20AA8B06E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFA16C54-6420-4CA8-B250-EADF06267DEF}">
   <dimension ref="B9:E120"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>